<commit_message>
update all PR Decoration files
</commit_message>
<xml_diff>
--- a/DOCs/sales-v3-tracker.xlsx
+++ b/DOCs/sales-v3-tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VDR000691\Documents\Tawn-Scripts\DOCs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11ED63D0-927B-4833-8E38-2BEF621C00DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8997F1F-EE90-4436-B956-D757896A915D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -544,6 +544,9 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -556,9 +559,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -835,13 +835,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -994,15 +994,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -1264,15 +1264,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -1460,23 +1460,23 @@
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="34.28515625" customWidth="1"/>
-    <col min="5" max="5" width="34.28515625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="34.28515625" style="15" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
     <col min="7" max="7" width="21.7109375" customWidth="1"/>
     <col min="8" max="8" width="127" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -1995,15 +1995,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">

</xml_diff>

<commit_message>
add updated powershell script
</commit_message>
<xml_diff>
--- a/DOCs/sales-v3-tracker.xlsx
+++ b/DOCs/sales-v3-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VDR000691\Documents\Tawn-Scripts\DOCs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58AF641-76A0-4732-84CB-0C04E9230CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE833870-ECF7-4E2E-BB30-7A47FBC90F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="118">
   <si>
     <t>Monorepo Split - Migration Dashboard (Tawuniya digital products)</t>
   </si>
@@ -388,6 +388,21 @@
   </si>
   <si>
     <t>Release Group</t>
+  </si>
+  <si>
+    <t>life-otp</t>
+  </si>
+  <si>
+    <t>dh-claims</t>
+  </si>
+  <si>
+    <t>acceptance-form</t>
+  </si>
+  <si>
+    <t>Job Configured</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -397,7 +412,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,6 +443,12 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -514,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -565,6 +586,9 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -577,6 +601,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -862,13 +889,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1021,15 +1048,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -1291,15 +1318,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -1484,7 +1511,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1494,20 +1521,20 @@
     <col min="5" max="5" width="34.28515625" style="15" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
     <col min="7" max="7" width="21.7109375" customWidth="1"/>
-    <col min="8" max="8" width="127" customWidth="1"/>
+    <col min="8" max="8" width="51" style="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -1532,7 +1559,7 @@
         <v>17</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1555,7 +1582,9 @@
       <c r="G4" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H4" s="9"/>
+      <c r="H4" s="10" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
@@ -1577,7 +1606,7 @@
       <c r="G5" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H5" s="9"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
@@ -1599,7 +1628,7 @@
       <c r="G6" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="9"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
@@ -1621,7 +1650,7 @@
       <c r="G7" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H7" s="9"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
@@ -1643,7 +1672,7 @@
       <c r="G8" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H8" s="9"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
@@ -1665,7 +1694,7 @@
       <c r="G9" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H9" s="9"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
@@ -1685,7 +1714,7 @@
       <c r="G10" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H10" s="9"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
@@ -1705,7 +1734,7 @@
       <c r="G11" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="9"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
@@ -1725,7 +1754,7 @@
       <c r="G12" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H12" s="9"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
@@ -1745,7 +1774,7 @@
       <c r="G13" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H13" s="9"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
@@ -1765,7 +1794,7 @@
       <c r="G14" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H14" s="9"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
@@ -1785,7 +1814,7 @@
       <c r="G15" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H15" s="9"/>
+      <c r="H15" s="10"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
@@ -1805,7 +1834,7 @@
       <c r="G16" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H16" s="9"/>
+      <c r="H16" s="10"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
@@ -1825,7 +1854,7 @@
       <c r="G17" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H17" s="9"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
@@ -1845,7 +1874,7 @@
       <c r="G18" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H18" s="9"/>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
@@ -1865,7 +1894,7 @@
       <c r="G19" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H19" s="9"/>
+      <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -1885,7 +1914,7 @@
       <c r="G20" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="9"/>
+      <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
@@ -1905,7 +1934,7 @@
       <c r="G21" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H21" s="9"/>
+      <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
@@ -1925,7 +1954,7 @@
       <c r="G22" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H22" s="9"/>
+      <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
@@ -1945,7 +1974,7 @@
       <c r="G23" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H23" s="9"/>
+      <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
@@ -1965,7 +1994,7 @@
       <c r="G24" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H24" s="9"/>
+      <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
@@ -1985,7 +2014,22 @@
       <c r="G25" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H25" s="9"/>
+      <c r="H25" s="10"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="18" t="s">
+        <v>115</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:H24" xr:uid="{00000000-0009-0000-0000-000003000000}">
@@ -2026,15 +2070,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">

</xml_diff>

<commit_message>
Add "webMethods-DEV-Server-Sync" and CRM SCAN files
</commit_message>
<xml_diff>
--- a/DOCs/sales-v3-tracker.xlsx
+++ b/DOCs/sales-v3-tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VDR000691\Documents\Tawn-Scripts\DOCs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9AE59C7-C405-417D-B723-E92FD939908C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76477A87-ACE6-4CA2-A84C-8F03A6008BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="112">
   <si>
     <t>Monorepo Split - Migration Dashboard (Tawuniya digital products)</t>
   </si>
@@ -111,9 +111,6 @@
     <t>motor</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Motor Retail (Individual)</t>
   </si>
   <si>
@@ -348,24 +345,12 @@
     <t>Payment Monorepo Migration Tracker  -  target repo: DH-Payment-V3</t>
   </si>
   <si>
-    <t>general-payment</t>
-  </si>
-  <si>
-    <t>Payment Gateway - General</t>
-  </si>
-  <si>
     <t>one-page-payment</t>
   </si>
   <si>
     <t>Payment Gateway - One Page</t>
   </si>
   <si>
-    <t>unified-payment</t>
-  </si>
-  <si>
-    <t>Payment Gateway - Unified</t>
-  </si>
-  <si>
     <t>Moataz Reda</t>
   </si>
   <si>
@@ -382,9 +367,6 @@
   </si>
   <si>
     <t>motor-upgrade</t>
-  </si>
-  <si>
-    <t>No pipeline</t>
   </si>
   <si>
     <t>Release Group</t>
@@ -452,7 +434,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -507,6 +489,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -535,7 +523,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -603,6 +591,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -983,7 +974,7 @@
       </c>
       <c r="B7" s="3">
         <f>COUNTA(Payment!A4:A6)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" s="3">
         <f>COUNTIF(Payment!B4:B6,"Yes")</f>
@@ -995,7 +986,7 @@
       </c>
       <c r="E7" s="4">
         <f>IF(B7=0,0,C7/B7)</f>
-        <v>0.33333333333333331</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1004,7 +995,7 @@
       </c>
       <c r="B8" s="6">
         <f>SUM(B4:B7)</f>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C8" s="6">
         <f>SUM(C4:C7)</f>
@@ -1016,7 +1007,7 @@
       </c>
       <c r="E8" s="7">
         <f>IF(B8=0,0,C8/B8)</f>
-        <v>0.95238095238095233</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1035,6 +1026,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <tabColor theme="9" tint="0.59999389629810485"/>
+  </sheetPr>
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1086,26 +1080,26 @@
         <v>19</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C4" s="10">
         <v>0</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
@@ -1117,29 +1111,29 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C7" s="10">
         <v>0</v>
@@ -1151,134 +1145,134 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G8" s="9"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C9" s="10">
         <v>0</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G9" s="9"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C10" s="10">
         <v>0</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G10" s="9"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C11" s="10">
         <v>0</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G11" s="9"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C12" s="10">
         <v>0</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G12" s="9"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C13" s="10">
         <v>0</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G13" s="9"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C14" s="10">
         <v>0</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G14" s="9"/>
     </row>
@@ -1305,6 +1299,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr>
+    <tabColor theme="9" tint="0.59999389629810485"/>
+  </sheetPr>
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1319,7 +1316,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -1353,134 +1350,134 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C4" s="10">
         <v>0</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G5" s="9"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C7" s="10">
         <v>0</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G7" s="9"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G8" s="9"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C9" s="10">
         <v>0</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G9" s="9"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C10" s="10">
         <v>0</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G10" s="9"/>
     </row>
@@ -1511,11 +1508,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <tabColor theme="9" tint="-0.249977111117893"/>
+  </sheetPr>
   <dimension ref="A1:H30"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="34.28515625" customWidth="1"/>
     <col min="5" max="5" width="34.28515625" style="15" customWidth="1"/>
@@ -1526,7 +1526,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
@@ -1550,7 +1550,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F3" s="12" t="s">
         <v>16</v>
@@ -1559,15 +1559,15 @@
         <v>17</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C4" s="10">
         <v>0</v>
@@ -1577,21 +1577,21 @@
         <v>1</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
@@ -1601,19 +1601,19 @@
         <v>1</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
@@ -1623,19 +1623,19 @@
         <v>1</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C7" s="10">
         <v>0</v>
@@ -1645,19 +1645,19 @@
         <v>2</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
@@ -1667,19 +1667,19 @@
         <v>2</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C9" s="10">
         <v>0</v>
@@ -1689,19 +1689,19 @@
         <v>2</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C10" s="10">
         <v>0</v>
@@ -1709,19 +1709,19 @@
       <c r="D10" s="9"/>
       <c r="E10" s="10"/>
       <c r="F10" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C11" s="10">
         <v>0</v>
@@ -1729,19 +1729,19 @@
       <c r="D11" s="9"/>
       <c r="E11" s="10"/>
       <c r="F11" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C12" s="10">
         <v>0</v>
@@ -1749,19 +1749,19 @@
       <c r="D12" s="9"/>
       <c r="E12" s="10"/>
       <c r="F12" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H12" s="10"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C13" s="10">
         <v>0</v>
@@ -1769,19 +1769,19 @@
       <c r="D13" s="9"/>
       <c r="E13" s="10"/>
       <c r="F13" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C14" s="10">
         <v>0</v>
@@ -1789,19 +1789,19 @@
       <c r="D14" s="9"/>
       <c r="E14" s="10"/>
       <c r="F14" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C15" s="10">
         <v>0</v>
@@ -1809,19 +1809,19 @@
       <c r="D15" s="9"/>
       <c r="E15" s="10"/>
       <c r="F15" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H15" s="10"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C16" s="10">
         <v>0</v>
@@ -1829,19 +1829,19 @@
       <c r="D16" s="9"/>
       <c r="E16" s="10"/>
       <c r="F16" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H16" s="10"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C17" s="10">
         <v>0</v>
@@ -1849,19 +1849,19 @@
       <c r="D17" s="9"/>
       <c r="E17" s="10"/>
       <c r="F17" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H17" s="10"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C18" s="10">
         <v>0</v>
@@ -1869,19 +1869,19 @@
       <c r="D18" s="9"/>
       <c r="E18" s="10"/>
       <c r="F18" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H18" s="10"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="H18" s="10"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>80</v>
-      </c>
       <c r="B19" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C19" s="10">
         <v>0</v>
@@ -1889,19 +1889,19 @@
       <c r="D19" s="9"/>
       <c r="E19" s="10"/>
       <c r="F19" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H19" s="10"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="H19" s="10"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
-        <v>82</v>
-      </c>
       <c r="B20" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C20" s="10">
         <v>0</v>
@@ -1909,19 +1909,19 @@
       <c r="D20" s="9"/>
       <c r="E20" s="10"/>
       <c r="F20" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C21" s="10">
         <v>0</v>
@@ -1929,19 +1929,19 @@
       <c r="D21" s="9"/>
       <c r="E21" s="10"/>
       <c r="F21" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C22" s="10">
         <v>0</v>
@@ -1949,19 +1949,19 @@
       <c r="D22" s="9"/>
       <c r="E22" s="10"/>
       <c r="F22" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C23" s="10">
         <v>0</v>
@@ -1969,19 +1969,19 @@
       <c r="D23" s="9"/>
       <c r="E23" s="10"/>
       <c r="F23" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C24" s="10">
         <v>0</v>
@@ -1989,19 +1989,19 @@
       <c r="D24" s="9"/>
       <c r="E24" s="10"/>
       <c r="F24" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C25" s="10">
         <v>0</v>
@@ -2009,26 +2009,26 @@
       <c r="D25" s="9"/>
       <c r="E25" s="10"/>
       <c r="F25" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H25" s="10"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2058,6 +2058,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2071,7 +2074,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -2104,65 +2107,41 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="10">
-        <v>0</v>
-      </c>
+      <c r="A4" s="9"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
       <c r="D4" s="9"/>
-      <c r="E4" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>111</v>
-      </c>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>101</v>
+      <c r="A5" s="25" t="s">
+        <v>98</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G5" s="9"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="10">
-        <v>0</v>
-      </c>
+      <c r="A6" s="9"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="9"/>
-      <c r="E6" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>111</v>
-      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G6" xr:uid="{00000000-0009-0000-0000-000004000000}"/>

</xml_diff>

<commit_message>
add Jenkins Syna files
</commit_message>
<xml_diff>
--- a/DOCs/sales-v3-tracker.xlsx
+++ b/DOCs/sales-v3-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VDR000691\Documents\Tawn-Scripts\DOCs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76477A87-ACE6-4CA2-A84C-8F03A6008BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220BD907-830C-40B1-B4CC-7AC155B0B292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -434,7 +434,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -495,6 +495,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -523,7 +529,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -580,6 +586,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -593,7 +602,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -880,13 +889,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
+      <c r="A1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1042,15 +1051,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -1315,15 +1324,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -1525,16 +1534,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -1697,7 +1706,7 @@
       <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="26" t="s">
         <v>57</v>
       </c>
       <c r="B10" s="10" t="s">
@@ -1737,7 +1746,7 @@
       <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="26" t="s">
         <v>61</v>
       </c>
       <c r="B12" s="10" t="s">
@@ -1757,7 +1766,7 @@
       <c r="H12" s="10"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="26" t="s">
         <v>63</v>
       </c>
       <c r="B13" s="10" t="s">
@@ -1877,7 +1886,7 @@
       <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="20" t="s">
         <v>79</v>
       </c>
       <c r="B19" s="10" t="s">
@@ -1897,7 +1906,7 @@
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="20" t="s">
         <v>81</v>
       </c>
       <c r="B20" s="10" t="s">
@@ -2073,15 +2082,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
@@ -2116,7 +2125,7 @@
       <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="20" t="s">
         <v>98</v>
       </c>
       <c r="B5" s="10" t="s">

</xml_diff>